<commit_message>
fix(plan-finca): revisión final aplicada — 0 B · 9 M · 26 m (9 M y 24 m arreglados)
M3: una sola regla (ninguna fecha en firme sin licencia; antes, reservas condicionadas con devolución
íntegra) en Word, contrato (cláusula Segunda bis), checklist, Excel, landing y correo. M6: la reserva
es «señal a cuenta del precio» regida por la tabla pactada (fuera las arras penitenciales). M4, M7:
notas de invierno e IVA del motor alineadas con la Tesorería y D4. M8: licencias y tasas sin IVA
(necesidad 360.503 €, sobrante 2.497 €). M1, M2, M5, M9 y 24 m de texto. Regenerados en el VPS:
ciclo.sh y D9 verdes, docx 6.906 palabras, contrato 150 párrafos, calculadora 588. Pendiente como deuda
común: PyG!G14 y Personal!C11 del motor, y la guía de equivalencias en Letter (las 53).

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-finca-eventos-bodas/calculadora-presupuesto-boda-evento-finca.xlsx
+++ b/astro-site/public/dl/plan-negocio-finca-eventos-bodas/calculadora-presupuesto-boda-evento-finca.xlsx
@@ -1410,7 +1410,7 @@
         <v>5399.625</v>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1">
+    <row r="64" ht="30" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
           <t>Importe retenido si cancela: tramo 5</t>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Último tramo, hasta el día del evento.</t>
+          <t>Último tramo, hasta el día del evento. Con particulares, el contrato descuenta de este importe los costes que la finca se ahorra por no celebrarlo.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="16" customHeight="1">
+    <row r="121" ht="30" customHeight="1">
       <c r="A121" s="4" t="inlineStr">
         <is>
           <t>Cancelación tramo 5: lo que retienes (% del total)</t>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Último mes o no presentación: el 100 %.</t>
+          <t>Último mes o no presentación: el 100 %. Con particulares, el contrato descuenta los costes que la finca se ahorra por no celebrarlo.</t>
         </is>
       </c>
     </row>

</xml_diff>